<commit_message>
Add Aircraft Maintenance Schedule (Phase 1): per-model recurring schedule, due/overdue warnings, Oil Change/50-Hour/Propeller Service/Avionics Check/AD Compliance coverage
</commit_message>
<xml_diff>
--- a/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
+++ b/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
@@ -16,10 +16,10 @@
     <sheet name="Summary" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Completed!$A$1:$E$30</definedName>
-    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'New Features (Backlog)'!$A$1:$G$8</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'On Hold'!$A$1:$E$16</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Pending!$A$1:$E$12</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Completed!$A$1:$E$36</definedName>
+    <definedName function="false" hidden="true" localSheetId="4" name="_xlnm._FilterDatabase" vbProcedure="false">'New Features (Backlog)'!$A$1:$G$9</definedName>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'On Hold'!$A$1:$E$15</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Pending!$A$1:$E$15</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="237">
   <si>
     <t xml:space="preserve">FlightPro Manager — Master Plan Tracker</t>
   </si>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">How this workbook is organized:</t>
   </si>
   <si>
-    <t xml:space="preserve">  •  Completed — shipped, committed, and (as of 2026-08-25) merged into production.</t>
+    <t xml:space="preserve">  •  Completed — shipped and delivered to the real machine; not every row is committed/merged into production yet (several 2026-08-26 items are delivered-but-uncommitted or committed-to-main-only as of this update) — see the handoff doc for each item's exact git state.</t>
   </si>
   <si>
     <t xml:space="preserve">  •  Pending — code is done and live, but not yet functionally verified. The two Urgent rows are security/accessibility fixes already live on production without having been tested.</t>
@@ -60,7 +60,7 @@
     <t xml:space="preserve">Suggested reading order for a 'what's next' conversation: check Pending first (two Urgent rows are live-on-production-untested and should happen before any new feature work), then compare the New Features sheet's Impact/Effort columns to pick the next build.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: compiled from claude/handoff-2026-08-18.md (the authoritative running log) and claude/next-steps-plan-2026-08-11.md (reconstructed backlog) as of 2026-08-25.</t>
+    <t xml:space="preserve">Source: compiled from the project's handoff doc (the authoritative running log, most recently /home/claude/handoff_work/final.md) as of 2026-08-26.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -315,6 +315,45 @@
     <t xml:space="preserve">main and production both at commit 4aefc5c, confirmed via real terminal output.</t>
   </si>
   <si>
+    <t xml:space="preserve">Medical Expiry null-input console error</t>
+  </si>
+  <si>
+    <t xml:space="preserve">React "value prop on input should not be null" — fixed missing || '' fallback in lib/store.ts's row mapper and StudentFormModal.tsx's populate-on-edit effect.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-26</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Broader icon-button aria-label coverage (item 38)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">11 files, 19 buttons — Edit/Delete pencil/trash icons across Admin Setup's 7 CRUD tabs plus Availability/Maintenance/Ground School Attendance pages now labeled with the row's own identifying name, not a generic "Edit"/"Delete". Closes the item deliberately deferred from session 7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial Weekly Off Day scheduling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New FTO Settings option covering all 3 real-world patterns: 1 weekly off, 2 weekly offs, or 1 weekly off + occurrence-based (e.g. every 2nd &amp; 4th Saturday, or every 1st/3rd/5th Saturday). Single shared getSchedulingBlockReason() used by every scheduling surface (BookingForm, ScheduleBoard, GroundSchoolCalendar, store).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial Weekly Off Day — Settings save not refreshing shared store</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Root cause: SettingsTab.tsx wrote settings to Supabase but never refreshed the Zustand store's cached ftoSettings — a pre-existing architectural gap affecting ANY setting change, not just the new feature. Found via user testing (29-08-2026 not blocked), fixed by refreshing the store after save.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BA Test Register write access narrowed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Removed admin/super_admin from BA_TEST_WRITE_ROLES — only safety_officer + operations can add/edit entries now; admin/super_admin retain view-only access via the existing REPORTS_VIEW_ROLES. Single source of truth (lib/permissions.ts) closes the gap across the UI and all 3 server routes at once.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aircraft Maintenance Schedule — Phase 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New per-model recurring maintenance schedule (engine TBO, Oil Change, 50/100-Hour Inspection, Annual Inspection, Propeller Service, Avionics Check, AD Compliance/ARC review — DGCA-researched, all 5 fleet models) driving: an Aircraft Model dropdown (with "Other" fallback), a non-blocking "Maintenance Due" warning panel, and staff-confirmed Set-Baseline / Create-Maintenance-Record actions. 4 SQL migrations + 13 code files. Phase 2 (hard-blocking bookings on overdue items) deliberately deferred to backlog.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Urgency</t>
   </si>
   <si>
@@ -399,6 +438,24 @@
     <t xml:space="preserve">Dashboard widget / Progress page / Instructor dashboard should all agree, now that the MULTI row exists.</t>
   </si>
   <si>
+    <t xml:space="preserve">Retest Partial Weekly Off Day feature</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm 29-08-2026 (2nd/4th Saturday rule) is now correctly blocked after the Settings-store-refresh fix — asked but not yet confirmed by the user.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Functionally test BA Test Register permission narrowing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confirm admin/super_admin can no longer add/edit BA entries (view-only) and safety_officer/operations still can, on the real logged-in app.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test Aircraft Maintenance Schedule Phase 1 (IN PROGRESS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">All 4 SQL migrations run 2026-08-26 — user is currently testing. Confirm: Maintenance Due panel shows the right items per aircraft; Set Baseline / Create Maintenance Record both save correctly; Aircraft Model dropdown populates from the schedule table with "Other" fallback working; logging a completion via the normal Log Maintenance screen (with Hobbs at Completion filled in) resets the matching item's due clock.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Why it's on hold</t>
   </si>
   <si>
@@ -414,15 +471,6 @@
     <t xml:space="preserve">Needs visual verification — not fixable blind in a sandbox with no deployed URL.</t>
   </si>
   <si>
-    <t xml:space="preserve">Broader icon-button aria-label coverage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Edit/delete pencil/trash icons beyond the Close-button scope already fixed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Scoped out of session 7 to the most acute gap (Close buttons) first.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Two more unhardened write paths</t>
   </si>
   <si>
@@ -639,6 +687,15 @@
     <t xml:space="preserve">No user demand signal yet beyond the original backlog line item — lowest apparent priority of the five backlog items.</t>
   </si>
   <si>
+    <t xml:space="preserve">Aircraft Maintenance Schedule — Phase 2 (hard-block bookings)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Auto-ground / block scheduling when a mandatory maintenance item goes overdue, instead of Phase 1's non-blocking warnings.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deliberately deferred by the user's own request until Phase 1 is confirmed working in practice; needs a decision on which items (if any) should be hard-blocking vs. warning-only, and how a false-positive baseline would be handled before an aircraft gets auto-grounded.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Plan Tracker — Summary</t>
   </si>
   <si>
@@ -663,22 +720,28 @@
     <t xml:space="preserve">Suggested next steps, in order</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Run the two Urgent items in Pending — session 7's security + accessibility fixes are live on production, untested. This is risk reduction, not new work, and should come first regardless of what's picked next.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2. Clear the rest of Pending with a normal testing pass (see the Pre-Handover Test Plan for the detailed step-by-step cases).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. For new feature work: Checkbox-style Requirements UI is the smallest, most self-contained backlog item and was already flagged as the natural next step — good first pick if you want visible progress fast.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4. The two DGCA implementation items (Incident Report, Maintenance Log) are High impact but blocked on you verifying the draft templates against the FTO's real paperwork first — worth doing that verification soon so they're unblocked whenever there's room.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5. Billing and Multi-FTO are both High-impact but Large-effort with no scoping done yet — good candidates for a dedicated scoping conversation before committing to either.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6. Mobile PWA installability and Multi-language are lower urgency — park until something above them is done.</t>
+    <t xml:space="preserve">1. Run the two Urgent items in Pending — session 7's security + accessibility fixes are live on production, still untested as of this update. This is risk reduction, not new work, and should come first regardless of what's picked next.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2. Finish testing the Aircraft Maintenance Schedule Phase 1 — all 4 SQL migrations are run, user is actively testing as of 2026-08-26 (see Pending). Once confirmed working, commit/push/merge and consider scoping Phase 2 (hard-blocking).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Retest Partial Weekly Off Day (29-08-2026 case) and functionally verify the BA Test Register permission narrowing — both shipped fixes awaiting confirmation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4. Clear the rest of Pending with a normal testing pass (see the Pre-Handover Test Plan for the detailed step-by-step cases).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5. For new feature work: Checkbox-style Requirements UI is still the smallest, most self-contained backlog item — good first pick if you want visible progress fast once the above testing is clear.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6. The two DGCA implementation items (Incident Report, Maintenance Log) are High impact but blocked on you verifying the draft templates against the FTO's real paperwork first — worth doing that verification soon so they're unblocked whenever there's room.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7. Billing and Multi-FTO are both High/Medium-impact but Large-effort with no scoping done yet — good candidates for a dedicated scoping conversation before committing to either.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8. Mobile PWA installability, Multi-language, and Aircraft Maintenance Schedule Phase 2 are lower urgency — park until something above them is done.</t>
   </si>
 </sst>
 </file>
@@ -879,8 +942,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -936,11 +1003,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -948,16 +1015,20 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -1296,56 +1367,56 @@
   <dimension ref="A1:A14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="105"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+    <row r="14" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -1365,528 +1436,630 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="n">
+    <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="n">
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="n">
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="n">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="n">
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="n">
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="6" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="n">
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="n">
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="n">
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="n">
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="C12" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="n">
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="n">
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="6" t="s">
+      <c r="C14" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="n">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="n">
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="n">
+    <row r="17" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B17" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C17" s="6" t="s">
+      <c r="C17" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="n">
+    <row r="18" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C18" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="n">
+    <row r="19" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="B19" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C19" s="6" t="s">
+      <c r="C19" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="n">
+    <row r="20" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="B20" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C20" s="6" t="s">
+      <c r="C20" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="n">
+    <row r="21" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C21" s="6" t="s">
+      <c r="C21" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="n">
+    <row r="22" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="B22" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="C22" s="6" t="s">
+      <c r="C22" s="7" t="s">
         <v>69</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="n">
+    <row r="23" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>72</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>73</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="6" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="n">
+    <row r="24" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="n">
+    <row r="25" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="5" t="n">
+    <row r="26" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="n">
+    <row r="27" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="n">
+    <row r="28" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="6" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="n">
+    <row r="29" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
+    <row r="30" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="6" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="B30" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="7" t="s">
         <v>92</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="E30" s="5" t="s">
+      <c r="E30" s="6" t="s">
         <v>77</v>
       </c>
     </row>
+    <row r="31" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="6" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C32" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C33" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="6" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C34" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="6" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C35" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="6" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>96</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E30"/>
+  <autoFilter ref="A1:E36"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -1903,222 +2076,273 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+      <c r="E1" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+      <c r="C2" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="E2" s="10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C3" s="8" t="s">
-        <v>98</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>99</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="C3" s="9" t="s">
+        <v>111</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="E3" s="10" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="C4" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>101</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+      <c r="C4" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="7" t="s">
-        <v>103</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>104</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="B5" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
+      <c r="B6" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>111</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
+      <c r="B7" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>123</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
+      <c r="B8" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="D9" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E9" s="11" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
+      <c r="B9" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C9" s="9" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
+      <c r="B10" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>130</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="D11" s="7" t="s">
+      <c r="B11" s="8" t="s">
         <v>119</v>
       </c>
-      <c r="E11" s="11" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
+      <c r="C11" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>120</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>121</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>109</v>
+      <c r="B12" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="9" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="8" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>137</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="E15" s="12" t="s">
+        <v>122</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E12"/>
+  <autoFilter ref="A1:E15"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2138,287 +2362,271 @@
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="55"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="55"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="E1" s="4" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="12" t="n">
+      <c r="E1" s="5" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="D2" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="12" t="n">
+      <c r="B2" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C2" s="14" t="s">
+        <v>143</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="n">
+      <c r="B3" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>146</v>
+      </c>
+      <c r="D3" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="E3" s="13" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>130</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="12" t="n">
+      <c r="B4" s="13" t="s">
+        <v>142</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>149</v>
+      </c>
+      <c r="D4" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="13" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="n">
+      <c r="B5" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>137</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E6" s="12" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="12" t="n">
+      <c r="B6" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>141</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="E7" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="12" t="n">
+      <c r="B7" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>144</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="12" t="n">
+      <c r="B8" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="13" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="D9" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="n">
+      <c r="B9" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>150</v>
-      </c>
-      <c r="D10" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="E10" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="n">
+      <c r="B10" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="C11" s="13" t="s">
+      <c r="B11" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="D11" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="E11" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="n">
+      <c r="C11" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="E12" s="12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="n">
+      <c r="B12" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C12" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="12" t="s">
+      <c r="B13" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>176</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="13" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="13" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="13" t="s">
-        <v>157</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>160</v>
-      </c>
-      <c r="D14" s="12" t="s">
-        <v>161</v>
-      </c>
-      <c r="E14" s="12" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>164</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="E15" s="12" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>167</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="E16" s="12" t="s">
-        <v>169</v>
-      </c>
-    </row>
+      <c r="C15" s="14" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:E16"/>
+  <autoFilter ref="A1:E15"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2435,203 +2643,226 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="C1" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="D1" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
+      <c r="C1" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="8" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
-        <v>175</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>176</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E2" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
+      <c r="B2" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>192</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E2" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="8" t="s">
-        <v>180</v>
-      </c>
-      <c r="C3" s="7" t="s">
-        <v>181</v>
-      </c>
-      <c r="D3" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="G3" s="7" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
+      <c r="B3" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
-        <v>184</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>185</v>
-      </c>
-      <c r="D4" s="7" t="s">
-        <v>182</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="F4" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="G4" s="7" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
+      <c r="B4" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="8" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>188</v>
-      </c>
-      <c r="D5" s="7" t="s">
-        <v>189</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="F5" s="7" t="s">
-        <v>178</v>
-      </c>
-      <c r="G5" s="7" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
+      <c r="B5" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="F5" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="8" t="s">
-        <v>191</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>192</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="F6" s="7" t="s">
+      <c r="B6" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>208</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="E6" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>212</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>193</v>
+      </c>
+      <c r="E7" s="11" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>195</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>196</v>
-      </c>
-      <c r="D7" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>178</v>
-      </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>214</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>199</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>177</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="F8" s="7" t="s">
+      <c r="E8" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>209</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="G8" s="7" t="s">
-        <v>201</v>
+      <c r="E9" s="11" t="s">
+        <v>194</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G8"/>
+  <autoFilter ref="A1:G9"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2648,127 +2879,137 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="14" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
-        <v>203</v>
-      </c>
-      <c r="B3" s="16" t="n">
-        <f aca="false">29</f>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
-        <v>204</v>
-      </c>
-      <c r="B4" s="16" t="n">
-        <f aca="false">11</f>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
-        <v>205</v>
-      </c>
-      <c r="B5" s="16" t="n">
-        <f aca="false">COUNTIF(Pending!E2:E12,"Urgent")</f>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="15" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>222</v>
+      </c>
+      <c r="B3" s="17" t="n">
+        <f aca="false">COUNT(Completed!A:A)</f>
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="16" t="s">
+        <v>223</v>
+      </c>
+      <c r="B4" s="17" t="n">
+        <f aca="false">COUNT(Pending!A:A)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="B5" s="17" t="n">
+        <f aca="false">COUNTIF(Pending!E:E,"Urgent")</f>
         <v>2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
-        <v>206</v>
-      </c>
-      <c r="B6" s="16" t="n">
-        <f aca="false">15</f>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
-        <v>207</v>
-      </c>
-      <c r="B7" s="16" t="n">
-        <f aca="false">7</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>208</v>
-      </c>
-      <c r="B8" s="16" t="n">
-        <f aca="false">COUNTIF('New Features (Backlog)'!E2:E8,"High")</f>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" s="17" t="n">
+        <f aca="false">COUNT('On Hold'!A:A)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="16" t="s">
+        <v>226</v>
+      </c>
+      <c r="B7" s="17" t="n">
+        <f aca="false">COUNT('New Features (Backlog)'!A:A)</f>
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="B8" s="17" t="n">
+        <f aca="false">COUNTIF('New Features (Backlog)'!E:E,"High")</f>
         <v>3</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="18" t="s">
-        <v>209</v>
-      </c>
-      <c r="B10" s="18"/>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="19" t="s">
+        <v>228</v>
+      </c>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
-        <v>210</v>
-      </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
+      <c r="A11" s="20" t="s">
+        <v>229</v>
+      </c>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="19" t="s">
-        <v>211</v>
-      </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
+      <c r="A12" s="20" t="s">
+        <v>230</v>
+      </c>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="19" t="s">
-        <v>212</v>
-      </c>
-      <c r="B13" s="19"/>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
+      <c r="A13" s="20" t="s">
+        <v>231</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>213</v>
-      </c>
-      <c r="B14" s="19"/>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
+      <c r="A14" s="20" t="s">
+        <v>232</v>
+      </c>
+      <c r="B14" s="20"/>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="B15" s="19"/>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
+      <c r="A15" s="20" t="s">
+        <v>233</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="19" t="s">
-        <v>215</v>
-      </c>
-      <c r="B16" s="19"/>
-      <c r="C16" s="19"/>
-      <c r="D16" s="19"/>
+      <c r="A16" s="20" t="s">
+        <v>234</v>
+      </c>
+      <c r="B16" s="20"/>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="21" t="s">
+        <v>236</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>

<commit_message>
Block saving an aircraft with an unrecognized Model; add CSV bulk import to Aircraft Maintenance Schedule
</commit_message>
<xml_diff>
--- a/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
+++ b/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="348" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="259">
   <si>
     <t xml:space="preserve">FlightPro Manager — Master Plan Tracker</t>
   </si>
@@ -42,7 +42,7 @@
     <t xml:space="preserve">How this workbook is organized:</t>
   </si>
   <si>
-    <t xml:space="preserve">  •  Completed — shipped and delivered to the real machine; not every row is committed/merged into production yet (several 2026-08-26 items are delivered-but-uncommitted or committed-to-main-only as of this update) — see the handoff doc for each item's exact git state.</t>
+    <t xml:space="preserve">  •  Completed — shipped and delivered to the real machine; the great majority is now committed, pushed, and merged into production — see the handoff doc for each item's exact git state.</t>
   </si>
   <si>
     <t xml:space="preserve">  •  Pending — code is done and live, but not yet functionally verified. The two Urgent rows are security/accessibility fixes already live on production without having been tested.</t>
@@ -60,7 +60,7 @@
     <t xml:space="preserve">Suggested reading order for a 'what's next' conversation: check Pending first (two Urgent rows are live-on-production-untested and should happen before any new feature work), then compare the New Features sheet's Impact/Effort columns to pick the next build.</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: compiled from the project's handoff doc (the authoritative running log, most recently /home/claude/handoff_work/final.md) as of 2026-08-26.</t>
+    <t xml:space="preserve">Source: compiled from the project's handoff doc (the authoritative running log, most recently claude/handoff-2026-08-27.md) as of 2026-08-27.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -354,6 +354,48 @@
     <t xml:space="preserve">New per-model recurring maintenance schedule (engine TBO, Oil Change, 50/100-Hour Inspection, Annual Inspection, Propeller Service, Avionics Check, AD Compliance/ARC review — DGCA-researched, all 5 fleet models) driving: an Aircraft Model dropdown (with "Other" fallback), a non-blocking "Maintenance Due" warning panel, and staff-confirmed Set-Baseline / Create-Maintenance-Record actions. 4 SQL migrations + 13 code files. Phase 2 (hard-blocking bookings on overdue items) deliberately deferred to backlog.</t>
   </si>
   <si>
+    <t xml:space="preserve">Aircraft Maintenance Schedule — Type/Model engine-type filtering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model dropdown now filtered by the selected engine Type (Single/Multi Engine); switching Type clears a now-mismatched Model. A model not yet mapped is shown for either Type so nothing becomes unselectable by omission.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aircraft Maintenance Schedule — fleet expansion to 9 models</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Added Cessna 152, Piper PA-28 Cherokee/Archer, Piper Archer DX, and Diamond DA40 with DGCA/manufacturer-researched schedule data (real sources, same discipline as the original 5 models).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type/Model engine-type mapping moved from hardcoded to DB-driven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New engine_type column on the schedule-template table, with an Admin Setup selector; adding or changing a model's engine type no longer needs a code change/redeploy — closes the last hardcoded-list gap in this feature.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aircraft Maintenance Schedule Phase 1 + fleet expansion committed, pushed, and merged into production</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Two commits (b1a5bd8, 819baef), both independently verified against GitHub. Merged to production before all testing was complete, per the user's explicit informed call.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UX / Data integrity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aircraft Model "Other (custom)" now warns and blocks Save instead of accepting free text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User's own suggestion: a custom Model that doesn't match a schedule template silently broke Maintenance Due tracking (the exact bug found earlier). Picking "Other" in both AircraftFormModal.tsx and AircraftSetupTab.tsx now shows an inline warning naming the current value (if any) and disables Save, pointing the admin at Admin Setup &gt; Aircraft Maintenance Schedule; a "Refresh list" button lets them pick the newly-added model without closing the form. Free text is kept ONLY as a bootstrap fallback for the (currently hypothetical) case of an empty schedule-template table. tsc clean, eslint introduces zero new issues (verified against the pre-edit baseline). Delivered to the real machine, confirmed byte-for-byte — not yet committed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aircraft Maintenance Schedule — CSV bulk import (Download Template / Upload CSV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User's request: adding schedule items one at a time was too slow for onboarding a new aircraft type's whole schedule. Added a Download Template / Upload CSV pair to the Admin Setup tab, mirroring ExercisesTab.tsx's existing CSV pattern (same papaparse library, same Append + skip-duplicates rule, no new dependency). Reuses the existing secured bulk-insert path in /api/admin/config/[table]/route.ts (already supported an array body) — no API changes needed. CSV rows can span multiple aircraft models in one upload, not just the currently-selected one. Client-side validates interval_type, interval_value, and engine_type before submitting (the DB CHECK constraints would otherwise fail the WHOLE batch on one bad row, since it's a single insert call) and pre-dedupes against the table's own unique(aircraft_model, item_name) constraint. tsc clean; eslint confirmed zero new issues via before/after diff against the unedited baseline. Delivered to the real machine, confirmed byte-for-byte — not yet committed.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Urgency</t>
   </si>
   <si>
@@ -453,7 +495,19 @@
     <t xml:space="preserve">Test Aircraft Maintenance Schedule Phase 1 (IN PROGRESS)</t>
   </si>
   <si>
-    <t xml:space="preserve">All 4 SQL migrations run 2026-08-26 — user is currently testing. Confirm: Maintenance Due panel shows the right items per aircraft; Set Baseline / Create Maintenance Record both save correctly; Aircraft Model dropdown populates from the schedule table with "Other" fallback working; logging a completion via the normal Log Maintenance screen (with Hobbs at Completion filled in) resets the matching item's due clock.</t>
+    <t xml:space="preserve">Confirmed working: Admin Setup schedule tab (9 models, Engine Type selector), Add/Edit Aircraft Type/Model filtering (incl. "Other (custom)" fallback and the pre-existing-aircraft Model re-pick), and the Maintenance Due panel's own Set Baseline / Create Maintenance Record buttons. Still needs a deliberate test: logging a completion through the normal "Log Maintenance" screen (not the Due panel's own buttons) — Type = Oil Change or similar, Status = Completed, Hobbs at Completion filled in — confirm the matching Due-panel item resets. This is the exact path the earlier item-name-mismatch bug was found and fixed in, so worth exercising deliberately rather than assuming it still works.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">General regression pass over the rest of the app</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Booking, Flight Records, Ground School, and the other Admin Setup tabs — nothing in this session's Aircraft Maintenance Schedule work should have touched them, but worth a normal-use sanity check now that everything (schedule feature, Type/Model filtering, fleet expansion, DB-driven engine type) is live on production.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test "Other (custom)" Model warn-and-block behavior</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add/Edit Aircraft, both AircraftFormModal.tsx and the Admin Setup Aircraft tab: pick "Other (custom)…", confirm the warning shows and Save/Add is disabled; add the model via Admin Setup &gt; Aircraft Maintenance Schedule, click "Refresh list", confirm it now appears and can be picked and saved. Also edit an aircraft with a legacy unmatched Model and confirm the same warning/block appears until it's re-picked.</t>
   </si>
   <si>
     <t xml:space="preserve">Why it's on hold</t>
@@ -696,6 +750,18 @@
     <t xml:space="preserve">Deliberately deferred by the user's own request until Phase 1 is confirmed working in practice; needs a decision on which items (if any) should be hard-blocking vs. warning-only, and how a false-positive baseline would be handled before an aircraft gets auto-grounded.</t>
   </si>
   <si>
+    <t xml:space="preserve">One-time "unrecognized Model" admin banner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A banner/flag (e.g. on Admin Setup or the Aircraft list) when N aircraft have a Model value that doesn't match any maintenance schedule template, with a one-click path to the affected aircraft's Edit form to re-pick the correct Model from the dropdown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Small</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-27 update: new aircraft can no longer be created/saved with an unrecognized Model at all (see Completed) — this item now only covers EXISTING aircraft that predate that fix (or were saved before the DB-driven engine_type migration). Lower priority than originally scoped, since the main failure mode is now closed at the point of entry.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Plan Tracker — Summary</t>
   </si>
   <si>
@@ -723,7 +789,7 @@
     <t xml:space="preserve">1. Run the two Urgent items in Pending — session 7's security + accessibility fixes are live on production, still untested as of this update. This is risk reduction, not new work, and should come first regardless of what's picked next.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Finish testing the Aircraft Maintenance Schedule Phase 1 — all 4 SQL migrations are run, user is actively testing as of 2026-08-26 (see Pending). Once confirmed working, commit/push/merge and consider scoping Phase 2 (hard-blocking).</t>
+    <t xml:space="preserve">2. Aircraft Maintenance Schedule Phase 1 + fleet expansion are now committed, pushed, and merged into production (2026-08-27). One targeted test remains — logging a completion via the normal Log Maintenance screen with Hobbs at Completion — plus a general regression pass over the rest of the app (see Pending). Once clear, consider scoping Phase 2 (hard-blocking bookings).</t>
   </si>
   <si>
     <t xml:space="preserve">3. Retest Partial Weekly Off Day (29-08-2026 case) and functionally verify the BA Test Register permission narrowing — both shipped fixes awaiting confirmation.</t>
@@ -1436,7 +1502,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -2056,6 +2122,108 @@
       </c>
       <c r="E36" s="6" t="s">
         <v>96</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C37" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C38" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="C39" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="6" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="C40" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C41" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="6" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2076,7 +2244,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -2100,7 +2268,7 @@
         <v>13</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>107</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2111,13 +2279,13 @@
         <v>15</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>108</v>
+        <v>122</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>109</v>
+        <v>123</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2128,13 +2296,13 @@
         <v>25</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>111</v>
+        <v>125</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>110</v>
+        <v>124</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2145,13 +2313,13 @@
         <v>81</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>114</v>
+        <v>128</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2159,16 +2327,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>118</v>
+        <v>132</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2176,16 +2344,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>120</v>
+        <v>134</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>121</v>
+        <v>135</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2193,16 +2361,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>123</v>
+        <v>137</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>124</v>
+        <v>138</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2210,16 +2378,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>125</v>
+        <v>139</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>126</v>
+        <v>140</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2227,16 +2395,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>127</v>
+        <v>141</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2244,16 +2412,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>129</v>
+        <v>143</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2261,16 +2429,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>131</v>
+        <v>145</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2278,16 +2446,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>133</v>
+        <v>147</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>134</v>
+        <v>148</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2295,16 +2463,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="D13" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="E13" s="12" t="s">
         <v>136</v>
-      </c>
-      <c r="E13" s="12" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2312,16 +2480,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>138</v>
+        <v>152</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2329,16 +2497,50 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>119</v>
+        <v>133</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>139</v>
+        <v>153</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>140</v>
+        <v>154</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>122</v>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="8" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C16" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="8" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="E17" s="12" t="s">
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2383,7 +2585,7 @@
         <v>13</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>141</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2391,16 +2593,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>144</v>
+        <v>162</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>145</v>
+        <v>163</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2411,13 +2613,13 @@
         <v>15</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>146</v>
+        <v>164</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>148</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2425,16 +2627,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>142</v>
+        <v>160</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2442,16 +2644,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>153</v>
+        <v>171</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>155</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2459,16 +2661,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>157</v>
+        <v>175</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>158</v>
+        <v>176</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2476,16 +2678,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>160</v>
+        <v>178</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>161</v>
+        <v>179</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>162</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2493,16 +2695,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>163</v>
+        <v>181</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>164</v>
+        <v>182</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>165</v>
+        <v>183</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2510,16 +2712,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>166</v>
+        <v>184</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>167</v>
+        <v>185</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2527,16 +2729,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>168</v>
+        <v>186</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>169</v>
+        <v>187</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2544,16 +2746,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>152</v>
+        <v>170</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>170</v>
+        <v>188</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>171</v>
+        <v>189</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>159</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2561,16 +2763,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>173</v>
+        <v>191</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2578,16 +2780,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>172</v>
+        <v>190</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>177</v>
+        <v>195</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>178</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2595,16 +2797,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>179</v>
+        <v>197</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>180</v>
+        <v>198</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>181</v>
+        <v>199</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>182</v>
+        <v>200</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2612,16 +2814,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>156</v>
+        <v>174</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>183</v>
+        <v>201</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>184</v>
+        <v>202</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>185</v>
+        <v>203</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2643,7 +2845,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -2662,19 +2864,19 @@
         <v>30</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2682,22 +2884,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>191</v>
+        <v>209</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>192</v>
+        <v>210</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2705,22 +2907,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>196</v>
+        <v>214</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2728,22 +2930,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2751,22 +2953,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>203</v>
+        <v>221</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>204</v>
+        <v>222</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>205</v>
+        <v>223</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>206</v>
+        <v>224</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2774,22 +2976,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>207</v>
+        <v>225</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>208</v>
+        <v>226</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>115</v>
+        <v>129</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>210</v>
+        <v>228</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2797,22 +2999,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>230</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="E7" s="11" t="s">
         <v>212</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>193</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>194</v>
-      </c>
       <c r="F7" s="8" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>213</v>
+        <v>231</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2820,22 +3022,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>214</v>
+        <v>232</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>215</v>
+        <v>233</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>216</v>
+        <v>234</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>209</v>
+        <v>227</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>217</v>
+        <v>235</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2843,22 +3045,45 @@
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>218</v>
+        <v>236</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>219</v>
+        <v>237</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>193</v>
+        <v>211</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>220</v>
+        <v>238</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>239</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>234</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -2888,30 +3113,30 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
       <c r="B3" s="17" t="n">
         <f aca="false">COUNT(Completed!A:A)</f>
-        <v>35</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>223</v>
+        <v>245</v>
       </c>
       <c r="B4" s="17" t="n">
         <f aca="false">COUNT(Pending!A:A)</f>
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>224</v>
+        <v>246</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Pending!E:E,"Urgent")</f>
@@ -2920,7 +3145,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>225</v>
+        <v>247</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">COUNT('On Hold'!A:A)</f>
@@ -2929,16 +3154,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNT('New Features (Backlog)'!A:A)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">COUNTIF('New Features (Backlog)'!E:E,"High")</f>
@@ -2947,7 +3172,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>228</v>
+        <v>250</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
@@ -2955,7 +3180,7 @@
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -2963,7 +3188,7 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -2971,7 +3196,7 @@
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="B13" s="20"/>
       <c r="C13" s="20"/>
@@ -2979,7 +3204,7 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
@@ -2987,7 +3212,7 @@
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -2995,7 +3220,7 @@
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>234</v>
+        <v>256</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
@@ -3003,12 +3228,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>235</v>
+        <v>257</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>236</v>
+        <v>258</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added ticketing for safety incedents
</commit_message>
<xml_diff>
--- a/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
+++ b/docs/FlightPro_Manager_Master_Plan_Tracker.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="259">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="262">
   <si>
     <t xml:space="preserve">FlightPro Manager — Master Plan Tracker</t>
   </si>
@@ -387,33 +387,45 @@
     <t xml:space="preserve">Aircraft Model "Other (custom)" now warns and blocks Save instead of accepting free text</t>
   </si>
   <si>
-    <t xml:space="preserve">User's own suggestion: a custom Model that doesn't match a schedule template silently broke Maintenance Due tracking (the exact bug found earlier). Picking "Other" in both AircraftFormModal.tsx and AircraftSetupTab.tsx now shows an inline warning naming the current value (if any) and disables Save, pointing the admin at Admin Setup &gt; Aircraft Maintenance Schedule; a "Refresh list" button lets them pick the newly-added model without closing the form. Free text is kept ONLY as a bootstrap fallback for the (currently hypothetical) case of an empty schedule-template table. tsc clean, eslint introduces zero new issues (verified against the pre-edit baseline). Delivered to the real machine, confirmed byte-for-byte — not yet committed.</t>
+    <t xml:space="preserve">User's own suggestion: a custom Model that doesn't match a schedule template silently broke Maintenance Due tracking (the exact bug found earlier). Picking "Other" in both AircraftFormModal.tsx and AircraftSetupTab.tsx now shows an inline warning naming the current value (if any) and disables Save, pointing the admin at Admin Setup &gt; Aircraft Maintenance Schedule; a "Refresh list" button lets them pick the newly-added model without closing the form. Free text is kept ONLY as a bootstrap fallback for the (currently hypothetical) case of an empty schedule-template table. tsc clean, eslint introduces zero new issues (verified against the pre-edit baseline). Committed, pushed, and merged into production same day (commit e137913) — independently verified via git ls-remote: both main and production resolve to e1379130022e31a028f0d83ae4a6623c9f86d424.</t>
   </si>
   <si>
     <t xml:space="preserve">Aircraft Maintenance Schedule — CSV bulk import (Download Template / Upload CSV)</t>
   </si>
   <si>
-    <t xml:space="preserve">User's request: adding schedule items one at a time was too slow for onboarding a new aircraft type's whole schedule. Added a Download Template / Upload CSV pair to the Admin Setup tab, mirroring ExercisesTab.tsx's existing CSV pattern (same papaparse library, same Append + skip-duplicates rule, no new dependency). Reuses the existing secured bulk-insert path in /api/admin/config/[table]/route.ts (already supported an array body) — no API changes needed. CSV rows can span multiple aircraft models in one upload, not just the currently-selected one. Client-side validates interval_type, interval_value, and engine_type before submitting (the DB CHECK constraints would otherwise fail the WHOLE batch on one bad row, since it's a single insert call) and pre-dedupes against the table's own unique(aircraft_model, item_name) constraint. tsc clean; eslint confirmed zero new issues via before/after diff against the unedited baseline. Delivered to the real machine, confirmed byte-for-byte — not yet committed.</t>
+    <t xml:space="preserve">User's request: adding schedule items one at a time was too slow for onboarding a new aircraft type's whole schedule. Added a Download Template / Upload CSV pair to the Admin Setup tab, mirroring ExercisesTab.tsx's existing CSV pattern (same papaparse library, same Append + skip-duplicates rule, no new dependency). Reuses the existing secured bulk-insert path in /api/admin/config/[table]/route.ts (already supported an array body) — no API changes needed. CSV rows can span multiple aircraft models in one upload, not just the currently-selected one. Client-side validates interval_type, interval_value, and engine_type before submitting (the DB CHECK constraints would otherwise fail the WHOLE batch on one bad row, since it's a single insert call) and pre-dedupes against the table's own unique(aircraft_model, item_name) constraint. tsc clean; eslint confirmed zero new issues via before/after diff against the unedited baseline. Committed, pushed, and merged into production same day (commit e137913) — independently verified via git ls-remote: both main and production resolve to e1379130022e31a028f0d83ae4a6623c9f86d424.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test security-hardening round (automated portion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-21 security-hardening round (Admin Setup config-CRUD, Aircraft routes, Direct Exam Entry role gating) verified against LIVE PRODUCTION on 2026-08-28 via an automated Node.js script (scripts/security-hardening-test.mjs) covering all 7 test accounts (super_admin/admin/operations/maintenance/instructor/safety_officer/student): 114/114 automated checks passed, 0 failed. Every non-super_admin role correctly rejected (403) on all 8 Admin Setup config tables (POST tested per table; PATCH/DELETE role gating spot-checked on exercises as the representative table, since every table shares the identical one-line requireRole() check); a non-whitelisted body field was confirmed dropped rather than persisted. Aircraft routes correctly allow only admin/super_admin and reject every other role on POST/PATCH/DELETE. Direct Exam Entry correctly rejects every non-admin/instructor/super_admin role. All throwaway test rows self-cleaned with zero leftovers. Full report: scripts/security-test-reports/security-test-2026-08-28T08-24-16-652Z.{txt,html,json}. NOT covered by this automated pass (tracked separately in Pending): the Ground School Progress IDOR fix (client-side-only, needs a manual browser check with a second student account) and Direct Exam Entry's positive/allowed-role path (no safe automated cleanup path).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-28 (session 7 cont.)</t>
   </si>
   <si>
     <t xml:space="preserve">Urgency</t>
   </si>
   <si>
-    <t xml:space="preserve">Test security-hardening round</t>
-  </si>
-  <si>
-    <t xml:space="preserve">All 7 Admin Setup config-route tabs, Aircraft Setup, the IDOR fix, and the direct-exam-entry route — live on production, untested.</t>
+    <t xml:space="preserve">Manually verify remaining security-hardening items (IDOR + direct-exam positive path)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Automated round (all 8 Admin Setup config tables, Aircraft Setup, Direct Exam Entry negative path) passed 114/114 against production on 2026-08-28 — see Completed and scripts/security-test-reports/. Two items still need manual verification because they can't be safely automated: (1) the Ground School Progress IDOR fix (?student= URL override) — a client-side React guard with no server-observable difference, needs a real browser click-through with two distinct student accounts (only one dummy student account has been provided so far — a second is needed to actually exercise this); (2) the Direct Exam Entry route's positive/allowed-role path — no DELETE endpoint and no FK-existence check on the insert, so a successful call can't be cleanly undone; verify manually and clean up the resulting ground_school_enrollment row by hand if exercised.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test accessibility-hardening round</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escape closes all 15 modals; all 11 Close buttons announce correctly to a screen reader — live on production, untested.</t>
   </si>
   <si>
     <t xml:space="preserve">Urgent</t>
   </si>
   <si>
-    <t xml:space="preserve">Test accessibility-hardening round</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escape closes all 15 modals; all 11 Close buttons announce correctly to a screen reader — live on production, untested.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Test My Students instructor-only scoping</t>
   </si>
   <si>
@@ -441,9 +453,6 @@
     <t xml:space="preserve">Training-stage dropdown, student cards, students-list filter, target-hours consistency, Multi Engine/Simulator progress cards, Breath Analyser Register + Report end-to-end, instructor CPL server-side block, SPL/CPL issue-date fields.</t>
   </si>
   <si>
-    <t xml:space="preserve">Normal</t>
-  </si>
-  <si>
     <t xml:space="preserve">Permission override feature — no live test yet</t>
   </si>
   <si>
@@ -507,7 +516,7 @@
     <t xml:space="preserve">Test "Other (custom)" Model warn-and-block behavior</t>
   </si>
   <si>
-    <t xml:space="preserve">Add/Edit Aircraft, both AircraftFormModal.tsx and the Admin Setup Aircraft tab: pick "Other (custom)…", confirm the warning shows and Save/Add is disabled; add the model via Admin Setup &gt; Aircraft Maintenance Schedule, click "Refresh list", confirm it now appears and can be picked and saved. Also edit an aircraft with a legacy unmatched Model and confirm the same warning/block appears until it's re-picked.</t>
+    <t xml:space="preserve">LIVE ON PRODUCTION as of 2026-08-27 (commit e137913), untested. Add/Edit Aircraft, both AircraftFormModal.tsx and the Admin Setup Aircraft tab: pick "Other (custom)…", confirm the warning shows and Save/Add is disabled; add the model via Admin Setup &gt; Aircraft Maintenance Schedule, click "Refresh list", confirm it now appears and can be picked and saved. Also edit an aircraft with a legacy unmatched Model and confirm the same warning/block appears until it's re-picked.</t>
   </si>
   <si>
     <t xml:space="preserve">Why it's on hold</t>
@@ -786,7 +795,7 @@
     <t xml:space="preserve">Suggested next steps, in order</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Run the two Urgent items in Pending — session 7's security + accessibility fixes are live on production, still untested as of this update. This is risk reduction, not new work, and should come first regardless of what's picked next.</t>
+    <t xml:space="preserve">1. Accessibility testing (session 7's fixes are live on production, still untested) is now the one remaining Urgent item — run it next. Security's automated round passed 114/114 against production on 2026-08-28; only two narrow manual-only checks are left there (see Pending), no longer blocking.</t>
   </si>
   <si>
     <t xml:space="preserve">2. Aircraft Maintenance Schedule Phase 1 + fleet expansion are now committed, pushed, and merged into production (2026-08-27). One targeted test remains — logging a completion via the normal Log Maintenance screen with Hobbs at Completion — plus a general regression pass over the rest of the app (see Pending). Once clear, consider scoping Phase 2 (hard-blocking bookings).</t>
@@ -1502,7 +1511,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5"/>
@@ -2224,6 +2233,23 @@
       </c>
       <c r="E42" s="6" t="s">
         <v>109</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="90.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="6" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C43" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2268,7 +2294,7 @@
         <v>13</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2279,13 +2305,13 @@
         <v>15</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2296,13 +2322,13 @@
         <v>25</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2313,13 +2339,13 @@
         <v>81</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2327,16 +2353,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2344,16 +2370,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E6" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2361,16 +2387,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="E7" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2378,16 +2404,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2395,16 +2421,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="E9" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2412,16 +2438,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2429,16 +2455,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2446,16 +2472,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="E12" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2463,16 +2489,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="E13" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2480,16 +2506,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="D14" s="8" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="E14" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2497,16 +2523,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="D15" s="8" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="E15" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2514,16 +2540,16 @@
         <v>15</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D16" s="8" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="E16" s="12" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2531,16 +2557,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>133</v>
-      </c>
-      <c r="C17" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="D17" s="8" t="s">
-        <v>158</v>
-      </c>
-      <c r="E17" s="12" t="s">
-        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -2585,7 +2611,7 @@
         <v>13</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2593,16 +2619,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E2" s="13" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2613,13 +2639,13 @@
         <v>15</v>
       </c>
       <c r="C3" s="14" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="D3" s="13" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E3" s="13" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2627,16 +2653,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="C4" s="14" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="E4" s="13" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2644,16 +2670,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,16 +2687,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2678,16 +2704,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="E7" s="13" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2695,16 +2721,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="E8" s="13" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2712,16 +2738,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="E9" s="13" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2729,16 +2755,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="E10" s="13" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2746,16 +2772,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="E11" s="13" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2763,16 +2789,16 @@
         <v>11</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2780,16 +2806,16 @@
         <v>12</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2797,16 +2823,16 @@
         <v>13</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="C14" s="14" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2814,16 +2840,16 @@
         <v>14</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2864,19 +2890,19 @@
         <v>30</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="G1" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2884,22 +2910,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="G2" s="8" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2907,22 +2933,22 @@
         <v>2</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C3" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>219</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F3" s="8" t="s">
         <v>215</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>216</v>
-      </c>
-      <c r="E3" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>212</v>
-      </c>
       <c r="G3" s="8" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2930,22 +2956,22 @@
         <v>3</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="C4" s="8" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" s="8" t="s">
         <v>219</v>
       </c>
-      <c r="D4" s="8" t="s">
-        <v>216</v>
-      </c>
       <c r="E4" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2953,22 +2979,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2976,22 +3002,22 @@
         <v>5</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E6" s="7" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2999,22 +3025,22 @@
         <v>6</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="C7" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>215</v>
+      </c>
+      <c r="F7" s="8" t="s">
         <v>230</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>211</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>212</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>227</v>
-      </c>
       <c r="G7" s="8" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3022,22 +3048,22 @@
         <v>7</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="D8" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E8" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>235</v>
+        <v>238</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3045,22 +3071,22 @@
         <v>8</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3068,22 +3094,22 @@
         <v>9</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="E10" s="12" t="s">
-        <v>234</v>
+        <v>237</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -3113,21 +3139,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="B3" s="17" t="n">
         <f aca="false">COUNT(Completed!A:A)</f>
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B4" s="17" t="n">
         <f aca="false">COUNT(Pending!A:A)</f>
@@ -3136,16 +3162,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="18" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="B5" s="17" t="n">
         <f aca="false">COUNTIF(Pending!E:E,"Urgent")</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="B6" s="17" t="n">
         <f aca="false">COUNT('On Hold'!A:A)</f>
@@ -3154,7 +3180,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="B7" s="17" t="n">
         <f aca="false">COUNT('New Features (Backlog)'!A:A)</f>
@@ -3163,7 +3189,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="B8" s="17" t="n">
         <f aca="false">COUNTIF('New Features (Backlog)'!E:E,"High")</f>
@@ -3172,7 +3198,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="19" t="s">
-        <v>250</v>
+        <v>253</v>
       </c>
       <c r="B10" s="19"/>
       <c r="C10" s="19"/>
@@ -3180,7 +3206,7 @@
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3188,7 +3214,7 @@
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="20" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -3196,7 +3222,7 @@
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="20" t="s">
-        <v>253</v>
+        <v>256</v>
       </c>
       <c r="B13" s="20"/>
       <c r="C13" s="20"/>
@@ -3204,7 +3230,7 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
@@ -3212,7 +3238,7 @@
     </row>
     <row r="15" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="20" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -3220,7 +3246,7 @@
     </row>
     <row r="16" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="20" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
@@ -3228,12 +3254,12 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>